<commit_message>
added results for alt2
</commit_message>
<xml_diff>
--- a/output/model_outputs/consequence-table-results.xlsx
+++ b/output/model_outputs/consequence-table-results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ep-cpien\OneDrive\GitHub\ds-ibmr-2025\output\model_outputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/cpien_usbr_gov/Documents/Work/GitHub/ds-ibmr-2025/output/model_outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2FA008-11F2-488B-B7A9-CC80099DB012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{5D2FA008-11F2-488B-B7A9-CC80099DB012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{514A1AE0-0AFE-4050-9E09-605CDACAE31B}"/>
   <bookViews>
-    <workbookView xWindow="7740" yWindow="3735" windowWidth="21600" windowHeight="11385" xr2:uid="{A7661C25-C126-4A36-A066-8290E60841CC}"/>
+    <workbookView xWindow="-23025" yWindow="3030" windowWidth="19185" windowHeight="10395" xr2:uid="{A7661C25-C126-4A36-A066-8290E60841CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>alt1</t>
   </si>
   <si>
-    <t>status-quo</t>
-  </si>
-  <si>
     <t>altnum</t>
   </si>
   <si>
@@ -54,6 +51,15 @@
   </si>
   <si>
     <t>abundance</t>
+  </si>
+  <si>
+    <t>alt2</t>
+  </si>
+  <si>
+    <t>StatusQuo</t>
+  </si>
+  <si>
+    <t>MaxDS_Even</t>
   </si>
 </sst>
 </file>
@@ -425,27 +431,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE68A1C0-7DA8-48FE-8779-F43E6C5E9ADB}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>4</v>
-      </c>
-      <c r="D1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -453,10 +459,21 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>0.91516109999999995</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>1.0995562999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>